<commit_message>
Add analysis and visualization scripts for ablation study of PIEA module
- Created `analyze_rank_all.py` to compute average ranks of algorithms across multiple problems.
- Developed `make_heatmap.py` to generate a heatmap HTML report visualizing IGD results for different algorithm variants.
- Introduced `read_tables.py` to read and display information from Excel files containing experimental data.
- Added a markdown document `指标模式模块去留_决策建议.md` summarizing decision recommendations based on experimental findings.
- Generated an HTML report `指标模式消融_热力图.html` to present the heatmap of results.
</commit_message>
<xml_diff>
--- a/PlatEMO-master/PlatEMO/Algorithms/Multi-objective optimization/REMO_new2_AdaMao实验数据.xlsx
+++ b/PlatEMO-master/PlatEMO/Algorithms/Multi-objective optimization/REMO_new2_AdaMao实验数据.xlsx
@@ -1,31 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlatEMO-master\PlatEMO-master\PlatEMO\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649CFE7C-F3A9-476A-A6F9-A9C5487165AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{4ED4F6BE-E29A-466B-9D42-5C6C73B4A4C3}"/>
+    <workbookView windowWidth="29868" windowHeight="13380"/>
   </bookViews>
   <sheets>
     <sheet name="IGD" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="236">
   <si>
     <t>Problem</t>
   </si>
@@ -60,9 +62,6 @@
     <t>PIEA</t>
   </si>
   <si>
-    <t>REMO_MaO</t>
-  </si>
-  <si>
     <t>ABSAEA</t>
   </si>
   <si>
@@ -72,24 +71,6 @@
     <t>SSDE</t>
   </si>
   <si>
-    <t>REMO_C2RL</t>
-  </si>
-  <si>
-    <t>REMO_new2_confidence</t>
-  </si>
-  <si>
-    <t>REMO_new2_PIEA2</t>
-  </si>
-  <si>
-    <t>REMO_new2_PIEA3</t>
-  </si>
-  <si>
-    <t>R2_REMO</t>
-  </si>
-  <si>
-    <t>REMO_new2_PIEA</t>
-  </si>
-  <si>
     <t>R2AEA</t>
   </si>
   <si>
@@ -120,9 +101,6 @@
     <t>2.4207e+2 (7.32e+1) =</t>
   </si>
   <si>
-    <t>2.3656e+2 (5.56e+1) =</t>
-  </si>
-  <si>
     <t>3.6690e+2 (3.42e+1) -</t>
   </si>
   <si>
@@ -132,24 +110,6 @@
     <t>3.0456e+2 (3.26e+1) -</t>
   </si>
   <si>
-    <t>1.7948e+2 (3.95e+1) +</t>
-  </si>
-  <si>
-    <t>2.0330e+2 (3.09e+1) =</t>
-  </si>
-  <si>
-    <t>1.9268e+2 (4.06e+1) +</t>
-  </si>
-  <si>
-    <t>1.8852e+2 (4.02e+1) +</t>
-  </si>
-  <si>
-    <t>2.0907e+2 (5.81e+1) =</t>
-  </si>
-  <si>
-    <t>1.7715e+2 (2.75e+1) +</t>
-  </si>
-  <si>
     <t>2.7206e+2 (2.49e+1) -</t>
   </si>
   <si>
@@ -180,9 +140,6 @@
     <t>9.6871e-1 (5.69e-2) +</t>
   </si>
   <si>
-    <t>1.4179e+0 (1.25e-1) -</t>
-  </si>
-  <si>
     <t>1.5748e+0 (6.72e-2) -</t>
   </si>
   <si>
@@ -192,24 +149,6 @@
     <t>1.7149e+0 (2.10e-1) -</t>
   </si>
   <si>
-    <t>1.1391e+0 (1.16e-1) +</t>
-  </si>
-  <si>
-    <t>1.1207e+0 (1.06e-1) +</t>
-  </si>
-  <si>
-    <t>1.1296e+0 (7.78e-2) +</t>
-  </si>
-  <si>
-    <t>1.1211e+0 (7.69e-2) +</t>
-  </si>
-  <si>
-    <t>1.0339e+0 (9.01e-2) +</t>
-  </si>
-  <si>
-    <t>1.0657e+0 (7.51e-2) +</t>
-  </si>
-  <si>
     <t>1.4611e+0 (5.68e-2) -</t>
   </si>
   <si>
@@ -240,9 +179,6 @@
     <t>5.5459e+2 (1.06e+2) +</t>
   </si>
   <si>
-    <t>6.7587e+2 (1.57e+2) +</t>
-  </si>
-  <si>
     <t>1.3294e+3 (1.08e+2) -</t>
   </si>
   <si>
@@ -252,24 +188,6 @@
     <t>1.1125e+3 (9.60e+1) -</t>
   </si>
   <si>
-    <t>7.6281e+2 (1.47e+2) +</t>
-  </si>
-  <si>
-    <t>8.4532e+2 (1.21e+2) =</t>
-  </si>
-  <si>
-    <t>7.5313e+2 (1.14e+2) +</t>
-  </si>
-  <si>
-    <t>7.0641e+2 (1.35e+2) +</t>
-  </si>
-  <si>
-    <t>7.1970e+2 (1.22e+2) +</t>
-  </si>
-  <si>
-    <t>6.7579e+2 (1.61e+2) +</t>
-  </si>
-  <si>
     <t>5.6353e+2 (6.65e+1) +</t>
   </si>
   <si>
@@ -300,9 +218,6 @@
     <t>1.2452e+0 (4.05e-2) =</t>
   </si>
   <si>
-    <t>1.3965e+0 (1.40e-1) =</t>
-  </si>
-  <si>
     <t>1.7642e+0 (5.53e-2) -</t>
   </si>
   <si>
@@ -312,24 +227,6 @@
     <t>1.7453e+0 (1.01e-1) -</t>
   </si>
   <si>
-    <t>1.1462e+0 (9.89e-2) +</t>
-  </si>
-  <si>
-    <t>1.1051e+0 (6.13e-2) +</t>
-  </si>
-  <si>
-    <t>1.1286e+0 (9.51e-2) +</t>
-  </si>
-  <si>
-    <t>1.1297e+0 (8.75e-2) +</t>
-  </si>
-  <si>
-    <t>1.0652e+0 (7.68e-2) +</t>
-  </si>
-  <si>
-    <t>1.1515e+0 (1.20e-1) +</t>
-  </si>
-  <si>
     <t>1.5944e+0 (7.20e-2) -</t>
   </si>
   <si>
@@ -360,9 +257,6 @@
     <t>2.9016e-1 (3.54e-2) +</t>
   </si>
   <si>
-    <t>7.2818e-1 (1.62e-1) =</t>
-  </si>
-  <si>
     <t>9.8945e-1 (8.10e-2) -</t>
   </si>
   <si>
@@ -372,24 +266,6 @@
     <t>1.1966e+0 (2.08e-1) -</t>
   </si>
   <si>
-    <t>5.5558e-1 (9.61e-2) =</t>
-  </si>
-  <si>
-    <t>5.7817e-1 (1.15e-1) =</t>
-  </si>
-  <si>
-    <t>5.1054e-1 (1.10e-1) +</t>
-  </si>
-  <si>
-    <t>5.7371e-1 (1.04e-1) =</t>
-  </si>
-  <si>
-    <t>5.3441e-1 (1.04e-1) =</t>
-  </si>
-  <si>
-    <t>5.8526e-1 (1.13e-1) =</t>
-  </si>
-  <si>
     <t>9.8650e-1 (8.39e-2) -</t>
   </si>
   <si>
@@ -420,9 +296,6 @@
     <t>5.4851e+0 (1.81e+0) +</t>
   </si>
   <si>
-    <t>1.6025e+1 (1.02e+0) -</t>
-  </si>
-  <si>
     <t>1.7962e+1 (1.49e-1) -</t>
   </si>
   <si>
@@ -432,24 +305,6 @@
     <t>1.4291e+1 (1.06e+0) -</t>
   </si>
   <si>
-    <t>1.5116e+1 (9.51e-1) -</t>
-  </si>
-  <si>
-    <t>1.5505e+1 (9.45e-1) -</t>
-  </si>
-  <si>
-    <t>1.4887e+1 (9.56e-1) -</t>
-  </si>
-  <si>
-    <t>1.5215e+1 (1.21e+0) -</t>
-  </si>
-  <si>
-    <t>1.6247e+1 (8.26e-1) -</t>
-  </si>
-  <si>
-    <t>1.5004e+1 (9.95e-1) -</t>
-  </si>
-  <si>
     <t>1.3116e+1 (1.22e+0) =</t>
   </si>
   <si>
@@ -480,9 +335,6 @@
     <t>1.8588e+1 (5.79e+0) -</t>
   </si>
   <si>
-    <t>8.1038e+0 (1.60e+0) =</t>
-  </si>
-  <si>
     <t>2.9805e+1 (1.71e+0) -</t>
   </si>
   <si>
@@ -492,24 +344,6 @@
     <t>2.6289e+1 (3.16e+0) -</t>
   </si>
   <si>
-    <t>1.6537e+1 (2.15e+0) -</t>
-  </si>
-  <si>
-    <t>1.7006e+1 (2.21e+0) -</t>
-  </si>
-  <si>
-    <t>1.7496e+1 (2.65e+0) -</t>
-  </si>
-  <si>
-    <t>1.5552e+1 (2.28e+0) -</t>
-  </si>
-  <si>
-    <t>2.4083e+1 (3.37e+0) -</t>
-  </si>
-  <si>
-    <t>1.3181e+1 (1.74e+0) -</t>
-  </si>
-  <si>
     <t>6.0881e+0 (9.80e-1) +</t>
   </si>
   <si>
@@ -540,9 +374,6 @@
     <t>3.3433e+0 (4.96e-2) -</t>
   </si>
   <si>
-    <t>3.3401e+0 (7.60e-2) -</t>
-  </si>
-  <si>
     <t>3.4292e+0 (2.10e-2) -</t>
   </si>
   <si>
@@ -552,24 +383,6 @@
     <t>3.5457e+0 (6.99e-2) -</t>
   </si>
   <si>
-    <t>3.2237e+0 (7.40e-2) =</t>
-  </si>
-  <si>
-    <t>3.1971e+0 (5.15e-2) =</t>
-  </si>
-  <si>
-    <t>3.1882e+0 (7.50e-2) =</t>
-  </si>
-  <si>
-    <t>3.2093e+0 (7.56e-2) =</t>
-  </si>
-  <si>
-    <t>3.2638e+0 (1.09e-1) -</t>
-  </si>
-  <si>
-    <t>3.1921e+0 (7.34e-2) =</t>
-  </si>
-  <si>
     <t>3.2026e+0 (2.73e-2) =</t>
   </si>
   <si>
@@ -600,9 +413,6 @@
     <t>2.3710e+0 (4.69e-1) =</t>
   </si>
   <si>
-    <t>2.7846e+0 (9.81e-1) =</t>
-  </si>
-  <si>
     <t>3.9270e+0 (6.28e-1) -</t>
   </si>
   <si>
@@ -612,24 +422,6 @@
     <t>3.0031e+0 (3.68e-1) -</t>
   </si>
   <si>
-    <t>3.2140e+0 (8.27e-1) -</t>
-  </si>
-  <si>
-    <t>3.0160e+0 (7.65e-1) -</t>
-  </si>
-  <si>
-    <t>3.0386e+0 (9.65e-1) -</t>
-  </si>
-  <si>
-    <t>2.8212e+0 (9.35e-1) =</t>
-  </si>
-  <si>
-    <t>3.3655e+0 (8.89e-1) -</t>
-  </si>
-  <si>
-    <t>2.6115e+0 (8.51e-1) =</t>
-  </si>
-  <si>
     <t>2.1985e+0 (7.86e-2) =</t>
   </si>
   <si>
@@ -660,9 +452,6 @@
     <t>1.1823e+0 (1.49e-1) +</t>
   </si>
   <si>
-    <t>1.7255e+0 (6.29e-2) -</t>
-  </si>
-  <si>
     <t>1.6454e+0 (2.48e-2) -</t>
   </si>
   <si>
@@ -672,24 +461,6 @@
     <t>1.8544e+0 (1.21e-1) -</t>
   </si>
   <si>
-    <t>1.5758e+0 (1.24e-1) =</t>
-  </si>
-  <si>
-    <t>1.6278e+0 (9.66e-2) -</t>
-  </si>
-  <si>
-    <t>1.5874e+0 (1.41e-1) =</t>
-  </si>
-  <si>
-    <t>1.5726e+0 (1.32e-1) =</t>
-  </si>
-  <si>
-    <t>1.4792e+0 (1.13e-1) =</t>
-  </si>
-  <si>
-    <t>1.5881e+0 (1.23e-1) =</t>
-  </si>
-  <si>
     <t>1.6117e+0 (5.06e-2) -</t>
   </si>
   <si>
@@ -720,9 +491,6 @@
     <t>5.7766e+0 (5.86e-1) +</t>
   </si>
   <si>
-    <t>9.0666e+0 (1.20e+0) -</t>
-  </si>
-  <si>
     <t>9.4311e+0 (4.78e-1) -</t>
   </si>
   <si>
@@ -732,24 +500,6 @@
     <t>6.7307e+0 (3.76e-1) =</t>
   </si>
   <si>
-    <t>8.5117e+0 (9.77e-1) -</t>
-  </si>
-  <si>
-    <t>8.4820e+0 (1.09e+0) -</t>
-  </si>
-  <si>
-    <t>8.5685e+0 (1.00e+0) -</t>
-  </si>
-  <si>
-    <t>7.9965e+0 (8.75e-1) -</t>
-  </si>
-  <si>
-    <t>9.0895e+0 (1.08e+0) -</t>
-  </si>
-  <si>
-    <t>8.3981e+0 (8.68e-1) -</t>
-  </si>
-  <si>
     <t>5.8327e+0 (2.30e-1) +</t>
   </si>
   <si>
@@ -780,9 +530,6 @@
     <t>5.7544e+0 (2.59e-1) +</t>
   </si>
   <si>
-    <t>7.0406e+0 (8.02e-1) -</t>
-  </si>
-  <si>
     <t>7.0502e+0 (2.38e-1) -</t>
   </si>
   <si>
@@ -792,24 +539,6 @@
     <t>6.9422e+0 (2.92e-1) -</t>
   </si>
   <si>
-    <t>6.7837e+0 (3.96e-1) -</t>
-  </si>
-  <si>
-    <t>6.8042e+0 (3.87e-1) -</t>
-  </si>
-  <si>
-    <t>6.6559e+0 (6.29e-1) -</t>
-  </si>
-  <si>
-    <t>6.7492e+0 (5.54e-1) -</t>
-  </si>
-  <si>
-    <t>7.0027e+0 (3.83e-1) -</t>
-  </si>
-  <si>
-    <t>6.9547e+0 (5.41e-1) -</t>
-  </si>
-  <si>
     <t>6.6637e+0 (4.27e-1) -</t>
   </si>
   <si>
@@ -840,9 +569,6 @@
     <t>5.9360e+0 (4.03e-1) -</t>
   </si>
   <si>
-    <t>7.2520e+0 (7.89e-1) -</t>
-  </si>
-  <si>
     <t>7.4484e+0 (2.82e-1) -</t>
   </si>
   <si>
@@ -852,24 +578,6 @@
     <t>6.9416e+0 (5.72e-1) -</t>
   </si>
   <si>
-    <t>6.4319e+0 (5.44e-1) -</t>
-  </si>
-  <si>
-    <t>6.7177e+0 (3.68e-1) -</t>
-  </si>
-  <si>
-    <t>6.3609e+0 (5.59e-1) -</t>
-  </si>
-  <si>
-    <t>6.4777e+0 (3.44e-1) -</t>
-  </si>
-  <si>
-    <t>7.2639e+0 (5.29e-1) -</t>
-  </si>
-  <si>
-    <t>6.4946e+0 (5.54e-1) -</t>
-  </si>
-  <si>
     <t>5.2950e+0 (1.04e-1) -</t>
   </si>
   <si>
@@ -900,9 +608,6 @@
     <t>6.9139e+0 (5.04e-1) -</t>
   </si>
   <si>
-    <t>7.9351e+0 (7.68e-1) -</t>
-  </si>
-  <si>
     <t>7.7543e+0 (2.43e-1) -</t>
   </si>
   <si>
@@ -912,24 +617,6 @@
     <t>7.3905e+0 (4.99e-1) -</t>
   </si>
   <si>
-    <t>6.3162e+0 (7.18e-1) -</t>
-  </si>
-  <si>
-    <t>6.5722e+0 (5.89e-1) -</t>
-  </si>
-  <si>
-    <t>6.4548e+0 (5.94e-1) -</t>
-  </si>
-  <si>
-    <t>6.2561e+0 (4.61e-1) -</t>
-  </si>
-  <si>
-    <t>7.3340e+0 (6.68e-1) -</t>
-  </si>
-  <si>
-    <t>6.5141e+0 (6.08e-1) -</t>
-  </si>
-  <si>
     <t>6.5389e+0 (4.05e-1) -</t>
   </si>
   <si>
@@ -960,9 +647,6 @@
     <t>6.3573e+0 (4.99e-1) =</t>
   </si>
   <si>
-    <t>7.7199e+0 (5.84e-1) -</t>
-  </si>
-  <si>
     <t>7.5858e+0 (2.15e-1) -</t>
   </si>
   <si>
@@ -972,24 +656,6 @@
     <t>7.0975e+0 (6.76e-1) -</t>
   </si>
   <si>
-    <t>6.8364e+0 (4.41e-1) -</t>
-  </si>
-  <si>
-    <t>7.0029e+0 (3.87e-1) -</t>
-  </si>
-  <si>
-    <t>7.1033e+0 (4.14e-1) -</t>
-  </si>
-  <si>
-    <t>6.7417e+0 (4.11e-1) -</t>
-  </si>
-  <si>
-    <t>7.7781e+0 (3.90e-1) -</t>
-  </si>
-  <si>
-    <t>6.8336e+0 (5.08e-1) -</t>
-  </si>
-  <si>
     <t>5.5577e+0 (1.32e-1) +</t>
   </si>
   <si>
@@ -1020,9 +686,6 @@
     <t>5.7930e+0 (3.72e-1) +</t>
   </si>
   <si>
-    <t>7.9758e+0 (1.01e+0) -</t>
-  </si>
-  <si>
     <t>7.8392e+0 (3.11e-1) -</t>
   </si>
   <si>
@@ -1032,24 +695,6 @@
     <t>7.8878e+0 (3.68e-1) -</t>
   </si>
   <si>
-    <t>7.4530e+0 (8.21e-1) -</t>
-  </si>
-  <si>
-    <t>7.6240e+0 (8.11e-1) -</t>
-  </si>
-  <si>
-    <t>7.7990e+0 (8.87e-1) -</t>
-  </si>
-  <si>
-    <t>7.6262e+0 (6.88e-1) -</t>
-  </si>
-  <si>
-    <t>8.0407e+0 (6.59e-1) -</t>
-  </si>
-  <si>
-    <t>7.8865e+0 (7.37e-1) -</t>
-  </si>
-  <si>
     <t>6.6300e+0 (3.57e-1) +</t>
   </si>
   <si>
@@ -1077,25 +722,10 @@
     <t>8/4/4</t>
   </si>
   <si>
-    <t>1/10/5</t>
-  </si>
-  <si>
     <t>5/7/4</t>
   </si>
   <si>
     <t>0/15/1</t>
-  </si>
-  <si>
-    <t>4/9/3</t>
-  </si>
-  <si>
-    <t>2/10/4</t>
-  </si>
-  <si>
-    <t>5/9/2</t>
-  </si>
-  <si>
-    <t>3/10/3</t>
   </si>
   <si>
     <t>5/8/3</t>
@@ -1110,20 +740,18 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1131,24 +759,361 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3333E9"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1158,53 +1123,336 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1253,7 +1501,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1286,26 +1534,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1338,23 +1569,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1496,26 +1710,21 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{945E32F0-4EC2-48AF-BA76-1EB58F659F1D}">
-  <dimension ref="A1:X18"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:U18"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
-    <col min="2" max="5" width="6.77734375" customWidth="1"/>
-    <col min="6" max="24" width="22.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.7777777777778" customWidth="1"/>
+    <col min="2" max="5" width="6.77777777777778" customWidth="1"/>
+    <col min="6" max="24" width="22.7777777777778" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,31 +1776,13 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+    </row>
+    <row r="2" spans="1:21">
+      <c r="A2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="B2" s="1">
         <v>100</v>
@@ -1606,66 +1797,48 @@
         <v>300</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="2"/>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="B3" s="1">
         <v>100</v>
@@ -1680,66 +1853,48 @@
         <v>300</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>63</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="B4" s="1">
         <v>100</v>
@@ -1754,66 +1909,48 @@
         <v>300</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>83</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1">
         <v>100</v>
@@ -1828,66 +1965,48 @@
         <v>300</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="T5" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>103</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="S5" s="1"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="1"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21">
       <c r="A6" s="1" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="B6" s="1">
         <v>100</v>
@@ -1902,66 +2021,48 @@
         <v>300</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>123</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21">
       <c r="A7" s="1" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="B7" s="1">
         <v>100</v>
@@ -1976,66 +2077,48 @@
         <v>300</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>127</v>
+        <v>85</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>128</v>
+        <v>86</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>130</v>
+        <v>88</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="S7" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>143</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21">
       <c r="A8" s="1" t="s">
-        <v>144</v>
+        <v>95</v>
       </c>
       <c r="B8" s="1">
         <v>100</v>
@@ -2050,66 +2133,48 @@
         <v>300</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>145</v>
+        <v>96</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>146</v>
+        <v>97</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>150</v>
+        <v>101</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>151</v>
+        <v>102</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>152</v>
+        <v>103</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>154</v>
+        <v>104</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="S8" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="V8" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>163</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21">
       <c r="A9" s="1" t="s">
-        <v>164</v>
+        <v>108</v>
       </c>
       <c r="B9" s="1">
         <v>100</v>
@@ -2124,66 +2189,48 @@
         <v>300</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>165</v>
+        <v>109</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>166</v>
+        <v>110</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>168</v>
+        <v>112</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>169</v>
+        <v>113</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>170</v>
+        <v>114</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>171</v>
+        <v>115</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>173</v>
+        <v>117</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>175</v>
+        <v>118</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="S9" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>183</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21">
       <c r="A10" s="1" t="s">
-        <v>184</v>
+        <v>121</v>
       </c>
       <c r="B10" s="1">
         <v>100</v>
@@ -2198,66 +2245,48 @@
         <v>300</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>185</v>
+        <v>122</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>186</v>
+        <v>123</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>187</v>
+        <v>124</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>188</v>
+        <v>125</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>189</v>
+        <v>126</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>190</v>
+        <v>127</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>191</v>
+        <v>128</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>192</v>
+        <v>129</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>194</v>
+        <v>130</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>195</v>
+        <v>132</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="R10" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="V10" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="X10" s="1" t="s">
-        <v>203</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21">
       <c r="A11" s="1" t="s">
-        <v>204</v>
+        <v>134</v>
       </c>
       <c r="B11" s="1">
         <v>100</v>
@@ -2272,66 +2301,48 @@
         <v>300</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>205</v>
+        <v>135</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>206</v>
+        <v>136</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>207</v>
+        <v>137</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>209</v>
+        <v>139</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>210</v>
+        <v>140</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>211</v>
+        <v>141</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>212</v>
+        <v>142</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>213</v>
+        <v>143</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>214</v>
+        <v>144</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>215</v>
+        <v>145</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="R11" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="T11" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="U11" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="V11" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="W11" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="X11" s="1" t="s">
-        <v>223</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21">
       <c r="A12" s="1" t="s">
-        <v>224</v>
+        <v>147</v>
       </c>
       <c r="B12" s="1">
         <v>100</v>
@@ -2346,66 +2357,48 @@
         <v>300</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>225</v>
+        <v>148</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>226</v>
+        <v>149</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>227</v>
+        <v>150</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>228</v>
+        <v>151</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>229</v>
+        <v>152</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>230</v>
+        <v>153</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>231</v>
+        <v>154</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>232</v>
+        <v>155</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>233</v>
+        <v>156</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>234</v>
+        <v>157</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>235</v>
+        <v>158</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="R12" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="S12" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="T12" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="U12" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="X12" s="1" t="s">
-        <v>243</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="S12" s="1"/>
+      <c r="T12" s="1"/>
+      <c r="U12" s="1"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21">
       <c r="A13" s="1" t="s">
-        <v>244</v>
+        <v>160</v>
       </c>
       <c r="B13" s="1">
         <v>100</v>
@@ -2420,66 +2413,48 @@
         <v>300</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>245</v>
+        <v>161</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>246</v>
+        <v>162</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>247</v>
+        <v>163</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>248</v>
+        <v>164</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>249</v>
+        <v>165</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>250</v>
+        <v>166</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>251</v>
+        <v>167</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>252</v>
+        <v>168</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>253</v>
+        <v>169</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>254</v>
+        <v>170</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>255</v>
+        <v>171</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="R13" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="S13" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="V13" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="W13" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="X13" s="1" t="s">
-        <v>263</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="S13" s="1"/>
+      <c r="T13" s="1"/>
+      <c r="U13" s="1"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21">
       <c r="A14" s="1" t="s">
-        <v>264</v>
+        <v>173</v>
       </c>
       <c r="B14" s="1">
         <v>100</v>
@@ -2494,66 +2469,48 @@
         <v>300</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>265</v>
+        <v>174</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>266</v>
+        <v>175</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>267</v>
+        <v>176</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>268</v>
+        <v>177</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>269</v>
+        <v>178</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>270</v>
+        <v>179</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>271</v>
+        <v>180</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>272</v>
+        <v>181</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>273</v>
+        <v>182</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>274</v>
+        <v>183</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="R14" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="S14" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="W14" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>283</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21">
       <c r="A15" s="1" t="s">
-        <v>284</v>
+        <v>186</v>
       </c>
       <c r="B15" s="1">
         <v>100</v>
@@ -2568,66 +2525,48 @@
         <v>300</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>285</v>
+        <v>187</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>286</v>
+        <v>188</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>287</v>
+        <v>189</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>288</v>
+        <v>190</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>289</v>
+        <v>191</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>290</v>
+        <v>192</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>291</v>
+        <v>193</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>292</v>
+        <v>194</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>293</v>
+        <v>195</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>295</v>
+        <v>196</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="V15" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="W15" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="X15" s="1" t="s">
-        <v>303</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21">
       <c r="A16" s="1" t="s">
-        <v>304</v>
+        <v>199</v>
       </c>
       <c r="B16" s="1">
         <v>100</v>
@@ -2642,66 +2581,48 @@
         <v>300</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>305</v>
+        <v>200</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>306</v>
+        <v>201</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>307</v>
+        <v>202</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>308</v>
+        <v>203</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>309</v>
+        <v>204</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>310</v>
+        <v>205</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>311</v>
+        <v>206</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>312</v>
+        <v>207</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>314</v>
+        <v>208</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>209</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>315</v>
+        <v>210</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>318</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="U16" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="V16" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="W16" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="X16" s="1" t="s">
-        <v>323</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21">
       <c r="A17" s="1" t="s">
-        <v>324</v>
+        <v>212</v>
       </c>
       <c r="B17" s="1">
         <v>100</v>
@@ -2716,134 +2637,98 @@
         <v>300</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>325</v>
+        <v>213</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>326</v>
+        <v>214</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>327</v>
+        <v>215</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>328</v>
+        <v>216</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>329</v>
+        <v>217</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>330</v>
+        <v>218</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>331</v>
+        <v>219</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>332</v>
+        <v>220</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>333</v>
+        <v>221</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>334</v>
+        <v>222</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>335</v>
+        <v>223</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="R17" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="V17" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="W17" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="X17" s="1" t="s">
-        <v>343</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21">
       <c r="A18" s="3" t="s">
-        <v>344</v>
+        <v>225</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
-      <c r="F18" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="N18" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="O18" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="P18" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="Q18" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="R18" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="S18" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="T18" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="U18" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="V18" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="W18" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="X18" s="4" t="s">
-        <v>359</v>
-      </c>
+      <c r="F18" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A18:E18"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>